<commit_message>
test: adapt cypress stubbing to new runner endpoints
Co-authored-by: Tristan Huet <tristan.huet@cosmotech.com>
</commit_message>
<xml_diff>
--- a/cypress/fixtures/customers_empty_unauthorized_fields.xlsx
+++ b/cypress/fixtures/customers_empty_unauthorized_fields.xlsx
@@ -234,7 +234,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F10"/>
-  <sheetFormatPr defaultColWidth="12.94140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.95703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12.76"/>
   </cols>
@@ -412,7 +412,8 @@
       <c r="B10" s="0" t="n">
         <v>56</v>
       </c>
-      <c r="C10" s="5" t="b">
+      <c r="C10" s="5" t="n">
+        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="D10" s="4" t="s">

</xml_diff>